<commit_message>
Last ATM + readme
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://epflch-my.sharepoint.com/personal/martina_baroffio_epfl_ch/Documents/EPFL/MA1/ML/ML4Science/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_49B9D71E964C440E62355476585DCE3A87458BAF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8333085E-90FA-4C27-9545-504AB8F6BB04}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_08C1AEB71759AA0F62355476585DCE3A874466E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3335836-0023-4678-AD19-6D4DE6904158}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="932" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1388" uniqueCount="126">
   <si>
     <t>Model</t>
   </si>
@@ -338,6 +338,66 @@
   </si>
   <si>
     <t>0.1636</t>
+  </si>
+  <si>
+    <t>{'svm__C': 0.1, 'svm__gamma': 'scale', 'svm__kernel': 'rbf'}</t>
+  </si>
+  <si>
+    <t>0.7330</t>
+  </si>
+  <si>
+    <t>0.1492</t>
+  </si>
+  <si>
+    <t>{'rf__max_depth': None, 'rf__max_features': 'sqrt', 'rf__min_samples_leaf': 2, 'rf__min_samples_split': 2, 'rf__n_estimators': 100}</t>
+  </si>
+  <si>
+    <t>{'rf__max_depth': None, 'rf__max_features': 'sqrt', 'rf__min_samples_leaf': 1, 'rf__min_samples_split': 10, 'rf__n_estimators': 500}</t>
+  </si>
+  <si>
+    <t>{'rf__max_depth': None, 'rf__max_features': 'log2', 'rf__min_samples_leaf': 4, 'rf__min_samples_split': 2, 'rf__n_estimators': 300}</t>
+  </si>
+  <si>
+    <t>{'rf__max_depth': None, 'rf__max_features': 'sqrt', 'rf__min_samples_leaf': 2, 'rf__min_samples_split': 2, 'rf__n_estimators': 500}</t>
+  </si>
+  <si>
+    <t>{'rf__max_depth': None, 'rf__max_features': 'sqrt', 'rf__min_samples_leaf': 2, 'rf__min_samples_split': 5, 'rf__n_estimators': 100}</t>
+  </si>
+  <si>
+    <t>{'rf__max_depth': None, 'rf__max_features': 'log2', 'rf__min_samples_leaf': 2, 'rf__min_samples_split': 2, 'rf__n_estimators': 500}</t>
+  </si>
+  <si>
+    <t>0.6736</t>
+  </si>
+  <si>
+    <t>0.1523</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 1.0, 'xgb__learning_rate': 0.01, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 500, 'xgb__subsample': 0.8}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.6, 'xgb__learning_rate': 0.1, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 300, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.6, 'xgb__learning_rate': 0.05, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 100, 'xgb__subsample': 1.0}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 1.0, 'xgb__learning_rate': 0.1, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 300, 'xgb__subsample': 0.8}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 0.8, 'xgb__learning_rate': 0.1, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 500, 'xgb__subsample': 0.8}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 1.0, 'xgb__learning_rate': 0.01, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 300, 'xgb__subsample': 0.6}</t>
+  </si>
+  <si>
+    <t>{'xgb__colsample_bytree': 1.0, 'xgb__learning_rate': 0.01, 'xgb__max_depth': 3, 'xgb__min_child_weight': 1, 'xgb__n_estimators': 300, 'xgb__subsample': 0.8}</t>
+  </si>
+  <si>
+    <t>0.6873</t>
+  </si>
+  <si>
+    <t>0.1743</t>
   </si>
 </sst>
 </file>
@@ -700,7 +760,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I304"/>
+  <dimension ref="A1:I454"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
@@ -7743,6 +7803,3474 @@
         <v>105</v>
       </c>
     </row>
+    <row r="305" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A305" t="s">
+        <v>14</v>
+      </c>
+      <c r="B305" t="s">
+        <v>15</v>
+      </c>
+      <c r="C305">
+        <v>0.69841269841269848</v>
+      </c>
+      <c r="D305">
+        <v>0.81818181818181812</v>
+      </c>
+      <c r="E305" t="s">
+        <v>16</v>
+      </c>
+      <c r="F305">
+        <v>2.5</v>
+      </c>
+      <c r="G305">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="306" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A306" t="s">
+        <v>14</v>
+      </c>
+      <c r="B306" t="s">
+        <v>15</v>
+      </c>
+      <c r="C306">
+        <v>0.75158730158730158</v>
+      </c>
+      <c r="D306">
+        <v>0.31818181818181818</v>
+      </c>
+      <c r="E306" t="s">
+        <v>16</v>
+      </c>
+      <c r="F306">
+        <v>2.5</v>
+      </c>
+      <c r="G306">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="307" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A307" t="s">
+        <v>14</v>
+      </c>
+      <c r="B307" t="s">
+        <v>15</v>
+      </c>
+      <c r="C307">
+        <v>0.75992063492063489</v>
+      </c>
+      <c r="D307">
+        <v>0.77272727272727271</v>
+      </c>
+      <c r="E307" t="s">
+        <v>16</v>
+      </c>
+      <c r="F307">
+        <v>2.5</v>
+      </c>
+      <c r="G307">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="308" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A308" t="s">
+        <v>14</v>
+      </c>
+      <c r="B308" t="s">
+        <v>15</v>
+      </c>
+      <c r="C308">
+        <v>0.54523809523809519</v>
+      </c>
+      <c r="D308">
+        <v>0.81818181818181812</v>
+      </c>
+      <c r="E308" t="s">
+        <v>16</v>
+      </c>
+      <c r="F308">
+        <v>2.5</v>
+      </c>
+      <c r="G308">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="309" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A309" t="s">
+        <v>14</v>
+      </c>
+      <c r="B309" t="s">
+        <v>15</v>
+      </c>
+      <c r="C309">
+        <v>0.79920634920634936</v>
+      </c>
+      <c r="D309">
+        <v>0.53030303030303028</v>
+      </c>
+      <c r="E309" t="s">
+        <v>16</v>
+      </c>
+      <c r="F309">
+        <v>2.5</v>
+      </c>
+      <c r="G309">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="310" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A310" t="s">
+        <v>14</v>
+      </c>
+      <c r="B310" t="s">
+        <v>15</v>
+      </c>
+      <c r="C310">
+        <v>0.57341269841269837</v>
+      </c>
+      <c r="D310">
+        <v>0.95454545454545459</v>
+      </c>
+      <c r="E310" t="s">
+        <v>16</v>
+      </c>
+      <c r="F310">
+        <v>2.5</v>
+      </c>
+      <c r="G310">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="311" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A311" t="s">
+        <v>14</v>
+      </c>
+      <c r="B311" t="s">
+        <v>15</v>
+      </c>
+      <c r="C311">
+        <v>0.57817460317460323</v>
+      </c>
+      <c r="D311">
+        <v>0.65151515151515149</v>
+      </c>
+      <c r="E311" t="s">
+        <v>16</v>
+      </c>
+      <c r="F311">
+        <v>2.5</v>
+      </c>
+      <c r="G311">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="312" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A312" t="s">
+        <v>14</v>
+      </c>
+      <c r="B312" t="s">
+        <v>15</v>
+      </c>
+      <c r="C312">
+        <v>0.77380952380952372</v>
+      </c>
+      <c r="D312">
+        <v>0.60606060606060597</v>
+      </c>
+      <c r="E312" t="s">
+        <v>16</v>
+      </c>
+      <c r="F312">
+        <v>2.5</v>
+      </c>
+      <c r="G312">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="313" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A313" t="s">
+        <v>14</v>
+      </c>
+      <c r="B313" t="s">
+        <v>15</v>
+      </c>
+      <c r="C313">
+        <v>0.69404761904761914</v>
+      </c>
+      <c r="D313">
+        <v>0.5757575757575758</v>
+      </c>
+      <c r="E313" t="s">
+        <v>16</v>
+      </c>
+      <c r="F313">
+        <v>2.5</v>
+      </c>
+      <c r="G313">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="314" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A314" t="s">
+        <v>14</v>
+      </c>
+      <c r="B314" t="s">
+        <v>15</v>
+      </c>
+      <c r="C314">
+        <v>0.67738095238095231</v>
+      </c>
+      <c r="D314">
+        <v>0.68181818181818188</v>
+      </c>
+      <c r="E314" t="s">
+        <v>16</v>
+      </c>
+      <c r="F314">
+        <v>2.5</v>
+      </c>
+      <c r="G314">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="315" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A315" t="s">
+        <v>14</v>
+      </c>
+      <c r="B315" t="s">
+        <v>106</v>
+      </c>
+      <c r="C315">
+        <v>0.5</v>
+      </c>
+      <c r="D315">
+        <v>0.5</v>
+      </c>
+      <c r="E315" t="s">
+        <v>16</v>
+      </c>
+      <c r="F315">
+        <v>2.5</v>
+      </c>
+      <c r="G315">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="316" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A316" t="s">
+        <v>14</v>
+      </c>
+      <c r="B316" t="s">
+        <v>15</v>
+      </c>
+      <c r="C316">
+        <v>0.79682539682539699</v>
+      </c>
+      <c r="D316">
+        <v>0.56060606060606055</v>
+      </c>
+      <c r="E316" t="s">
+        <v>16</v>
+      </c>
+      <c r="F316">
+        <v>2.5</v>
+      </c>
+      <c r="G316">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="317" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A317" t="s">
+        <v>14</v>
+      </c>
+      <c r="B317" t="s">
+        <v>15</v>
+      </c>
+      <c r="C317">
+        <v>0.56111111111111112</v>
+      </c>
+      <c r="D317">
+        <v>0.63636363636363635</v>
+      </c>
+      <c r="E317" t="s">
+        <v>16</v>
+      </c>
+      <c r="F317">
+        <v>2.5</v>
+      </c>
+      <c r="G317">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="318" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A318" t="s">
+        <v>14</v>
+      </c>
+      <c r="B318" t="s">
+        <v>15</v>
+      </c>
+      <c r="C318">
+        <v>0.59761904761904761</v>
+      </c>
+      <c r="D318">
+        <v>0.83333333333333326</v>
+      </c>
+      <c r="E318" t="s">
+        <v>16</v>
+      </c>
+      <c r="F318">
+        <v>2.5</v>
+      </c>
+      <c r="G318">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="319" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A319" t="s">
+        <v>14</v>
+      </c>
+      <c r="B319" t="s">
+        <v>15</v>
+      </c>
+      <c r="C319">
+        <v>0.72658730158730156</v>
+      </c>
+      <c r="D319">
+        <v>0.77272727272727271</v>
+      </c>
+      <c r="E319" t="s">
+        <v>16</v>
+      </c>
+      <c r="F319">
+        <v>2.5</v>
+      </c>
+      <c r="G319">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="320" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A320" t="s">
+        <v>14</v>
+      </c>
+      <c r="B320" t="s">
+        <v>15</v>
+      </c>
+      <c r="C320">
+        <v>0.60238095238095235</v>
+      </c>
+      <c r="D320">
+        <v>0.65151515151515149</v>
+      </c>
+      <c r="E320" t="s">
+        <v>16</v>
+      </c>
+      <c r="F320">
+        <v>2.5</v>
+      </c>
+      <c r="G320">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="321" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A321" t="s">
+        <v>14</v>
+      </c>
+      <c r="B321" t="s">
+        <v>15</v>
+      </c>
+      <c r="C321">
+        <v>0.73571428571428577</v>
+      </c>
+      <c r="D321">
+        <v>0.39393939393939392</v>
+      </c>
+      <c r="E321" t="s">
+        <v>16</v>
+      </c>
+      <c r="F321">
+        <v>2.5</v>
+      </c>
+      <c r="G321">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="322" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A322" t="s">
+        <v>14</v>
+      </c>
+      <c r="B322" t="s">
+        <v>15</v>
+      </c>
+      <c r="C322">
+        <v>0.598015873015873</v>
+      </c>
+      <c r="D322">
+        <v>0.90909090909090917</v>
+      </c>
+      <c r="E322" t="s">
+        <v>16</v>
+      </c>
+      <c r="F322">
+        <v>2.5</v>
+      </c>
+      <c r="G322">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="323" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A323" t="s">
+        <v>14</v>
+      </c>
+      <c r="B323" t="s">
+        <v>15</v>
+      </c>
+      <c r="C323">
+        <v>0.66190476190476188</v>
+      </c>
+      <c r="D323">
+        <v>0.48484848484848492</v>
+      </c>
+      <c r="E323" t="s">
+        <v>16</v>
+      </c>
+      <c r="F323">
+        <v>2.5</v>
+      </c>
+      <c r="G323">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="324" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A324" t="s">
+        <v>14</v>
+      </c>
+      <c r="B324" t="s">
+        <v>15</v>
+      </c>
+      <c r="C324">
+        <v>0.74722222222222223</v>
+      </c>
+      <c r="D324">
+        <v>0.60606060606060597</v>
+      </c>
+      <c r="E324" t="s">
+        <v>16</v>
+      </c>
+      <c r="F324">
+        <v>2.5</v>
+      </c>
+      <c r="G324">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="325" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A325" t="s">
+        <v>14</v>
+      </c>
+      <c r="B325" t="s">
+        <v>15</v>
+      </c>
+      <c r="C325">
+        <v>0.67301587301587296</v>
+      </c>
+      <c r="D325">
+        <v>0.86363636363636365</v>
+      </c>
+      <c r="E325" t="s">
+        <v>16</v>
+      </c>
+      <c r="F325">
+        <v>2.5</v>
+      </c>
+      <c r="G325">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="326" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A326" t="s">
+        <v>14</v>
+      </c>
+      <c r="B326" t="s">
+        <v>15</v>
+      </c>
+      <c r="C326">
+        <v>0.5984126984126984</v>
+      </c>
+      <c r="D326">
+        <v>0.81818181818181812</v>
+      </c>
+      <c r="E326" t="s">
+        <v>16</v>
+      </c>
+      <c r="F326">
+        <v>2.5</v>
+      </c>
+      <c r="G326">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="327" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A327" t="s">
+        <v>14</v>
+      </c>
+      <c r="B327" t="s">
+        <v>15</v>
+      </c>
+      <c r="C327">
+        <v>0.759920634920635</v>
+      </c>
+      <c r="D327">
+        <v>0.78787878787878785</v>
+      </c>
+      <c r="E327" t="s">
+        <v>16</v>
+      </c>
+      <c r="F327">
+        <v>2.5</v>
+      </c>
+      <c r="G327">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="328" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A328" t="s">
+        <v>14</v>
+      </c>
+      <c r="B328" t="s">
+        <v>15</v>
+      </c>
+      <c r="C328">
+        <v>0.73730158730158735</v>
+      </c>
+      <c r="D328">
+        <v>0.72727272727272729</v>
+      </c>
+      <c r="E328" t="s">
+        <v>16</v>
+      </c>
+      <c r="F328">
+        <v>2.5</v>
+      </c>
+      <c r="G328">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="329" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A329" t="s">
+        <v>14</v>
+      </c>
+      <c r="B329" t="s">
+        <v>15</v>
+      </c>
+      <c r="C329">
+        <v>0.73492063492063497</v>
+      </c>
+      <c r="D329">
+        <v>0.74242424242424243</v>
+      </c>
+      <c r="E329" t="s">
+        <v>16</v>
+      </c>
+      <c r="F329">
+        <v>2.5</v>
+      </c>
+      <c r="G329">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="330" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A330" t="s">
+        <v>14</v>
+      </c>
+      <c r="B330" t="s">
+        <v>15</v>
+      </c>
+      <c r="C330">
+        <v>0.79484126984126979</v>
+      </c>
+      <c r="D330">
+        <v>0.69696969696969702</v>
+      </c>
+      <c r="E330" t="s">
+        <v>16</v>
+      </c>
+      <c r="F330">
+        <v>2.5</v>
+      </c>
+      <c r="G330">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="331" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A331" t="s">
+        <v>14</v>
+      </c>
+      <c r="B331" t="s">
+        <v>15</v>
+      </c>
+      <c r="C331">
+        <v>0.57579365079365075</v>
+      </c>
+      <c r="D331">
+        <v>0.68181818181818188</v>
+      </c>
+      <c r="E331" t="s">
+        <v>16</v>
+      </c>
+      <c r="F331">
+        <v>2.5</v>
+      </c>
+      <c r="G331">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="332" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A332" t="s">
+        <v>14</v>
+      </c>
+      <c r="B332" t="s">
+        <v>15</v>
+      </c>
+      <c r="C332">
+        <v>0.68492063492063482</v>
+      </c>
+      <c r="D332">
+        <v>0.77272727272727271</v>
+      </c>
+      <c r="E332" t="s">
+        <v>16</v>
+      </c>
+      <c r="F332">
+        <v>2.5</v>
+      </c>
+      <c r="G332">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="333" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A333" t="s">
+        <v>14</v>
+      </c>
+      <c r="B333" t="s">
+        <v>15</v>
+      </c>
+      <c r="C333">
+        <v>0.7325396825396826</v>
+      </c>
+      <c r="D333">
+        <v>1</v>
+      </c>
+      <c r="E333" t="s">
+        <v>16</v>
+      </c>
+      <c r="F333">
+        <v>2.5</v>
+      </c>
+      <c r="G333">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="334" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A334" t="s">
+        <v>14</v>
+      </c>
+      <c r="B334" t="s">
+        <v>15</v>
+      </c>
+      <c r="C334">
+        <v>0.85873015873015868</v>
+      </c>
+      <c r="D334">
+        <v>0.86363636363636365</v>
+      </c>
+      <c r="E334" t="s">
+        <v>16</v>
+      </c>
+      <c r="F334">
+        <v>2.5</v>
+      </c>
+      <c r="G334">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="335" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A335" t="s">
+        <v>14</v>
+      </c>
+      <c r="B335" t="s">
+        <v>15</v>
+      </c>
+      <c r="C335">
+        <v>0.76428571428571423</v>
+      </c>
+      <c r="D335">
+        <v>0.86363636363636365</v>
+      </c>
+      <c r="E335" t="s">
+        <v>16</v>
+      </c>
+      <c r="F335">
+        <v>2.5</v>
+      </c>
+      <c r="G335">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="336" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A336" t="s">
+        <v>14</v>
+      </c>
+      <c r="B336" t="s">
+        <v>15</v>
+      </c>
+      <c r="C336">
+        <v>0.64960317460317463</v>
+      </c>
+      <c r="D336">
+        <v>0.90909090909090917</v>
+      </c>
+      <c r="E336" t="s">
+        <v>16</v>
+      </c>
+      <c r="F336">
+        <v>2.5</v>
+      </c>
+      <c r="G336">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="337" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A337" t="s">
+        <v>14</v>
+      </c>
+      <c r="B337" t="s">
+        <v>15</v>
+      </c>
+      <c r="C337">
+        <v>0.62817460317460316</v>
+      </c>
+      <c r="D337">
+        <v>0.60606060606060597</v>
+      </c>
+      <c r="E337" t="s">
+        <v>16</v>
+      </c>
+      <c r="F337">
+        <v>2.5</v>
+      </c>
+      <c r="G337">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="338" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A338" t="s">
+        <v>14</v>
+      </c>
+      <c r="B338" t="s">
+        <v>15</v>
+      </c>
+      <c r="C338">
+        <v>0.77896825396825398</v>
+      </c>
+      <c r="D338">
+        <v>0.68181818181818188</v>
+      </c>
+      <c r="E338" t="s">
+        <v>16</v>
+      </c>
+      <c r="F338">
+        <v>2.5</v>
+      </c>
+      <c r="G338">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="339" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A339" t="s">
+        <v>14</v>
+      </c>
+      <c r="B339" t="s">
+        <v>15</v>
+      </c>
+      <c r="C339">
+        <v>0.6869047619047618</v>
+      </c>
+      <c r="D339">
+        <v>0.81818181818181812</v>
+      </c>
+      <c r="E339" t="s">
+        <v>16</v>
+      </c>
+      <c r="F339">
+        <v>2.5</v>
+      </c>
+      <c r="G339">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="340" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A340" t="s">
+        <v>14</v>
+      </c>
+      <c r="B340" t="s">
+        <v>15</v>
+      </c>
+      <c r="C340">
+        <v>0.68571428571428561</v>
+      </c>
+      <c r="D340">
+        <v>0.90909090909090917</v>
+      </c>
+      <c r="E340" t="s">
+        <v>16</v>
+      </c>
+      <c r="F340">
+        <v>2.5</v>
+      </c>
+      <c r="G340">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="341" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A341" t="s">
+        <v>14</v>
+      </c>
+      <c r="B341" t="s">
+        <v>15</v>
+      </c>
+      <c r="C341">
+        <v>0.73849206349206353</v>
+      </c>
+      <c r="D341">
+        <v>0.81818181818181812</v>
+      </c>
+      <c r="E341" t="s">
+        <v>16</v>
+      </c>
+      <c r="F341">
+        <v>2.5</v>
+      </c>
+      <c r="G341">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="342" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A342" t="s">
+        <v>14</v>
+      </c>
+      <c r="B342" t="s">
+        <v>15</v>
+      </c>
+      <c r="C342">
+        <v>0.64960317460317463</v>
+      </c>
+      <c r="D342">
+        <v>0.77272727272727271</v>
+      </c>
+      <c r="E342" t="s">
+        <v>16</v>
+      </c>
+      <c r="F342">
+        <v>2.5</v>
+      </c>
+      <c r="G342">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="343" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A343" t="s">
+        <v>14</v>
+      </c>
+      <c r="B343" t="s">
+        <v>15</v>
+      </c>
+      <c r="C343">
+        <v>0.78214285714285714</v>
+      </c>
+      <c r="D343">
+        <v>0.56060606060606055</v>
+      </c>
+      <c r="E343" t="s">
+        <v>16</v>
+      </c>
+      <c r="F343">
+        <v>2.5</v>
+      </c>
+      <c r="G343">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="344" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A344" t="s">
+        <v>14</v>
+      </c>
+      <c r="B344" t="s">
+        <v>15</v>
+      </c>
+      <c r="C344">
+        <v>0.54603174603174598</v>
+      </c>
+      <c r="D344">
+        <v>0.86363636363636365</v>
+      </c>
+      <c r="E344" t="s">
+        <v>16</v>
+      </c>
+      <c r="F344">
+        <v>2.5</v>
+      </c>
+      <c r="G344">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="345" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A345" t="s">
+        <v>14</v>
+      </c>
+      <c r="B345" t="s">
+        <v>15</v>
+      </c>
+      <c r="C345">
+        <v>0.64047619047619042</v>
+      </c>
+      <c r="D345">
+        <v>0.90909090909090917</v>
+      </c>
+      <c r="E345" t="s">
+        <v>16</v>
+      </c>
+      <c r="F345">
+        <v>2.5</v>
+      </c>
+      <c r="G345">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="346" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A346" t="s">
+        <v>14</v>
+      </c>
+      <c r="B346" t="s">
+        <v>15</v>
+      </c>
+      <c r="C346">
+        <v>0.85793650793650789</v>
+      </c>
+      <c r="D346">
+        <v>0.81818181818181812</v>
+      </c>
+      <c r="E346" t="s">
+        <v>16</v>
+      </c>
+      <c r="F346">
+        <v>2.5</v>
+      </c>
+      <c r="G346">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="347" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A347" t="s">
+        <v>14</v>
+      </c>
+      <c r="B347" t="s">
+        <v>15</v>
+      </c>
+      <c r="C347">
+        <v>0.63809523809523805</v>
+      </c>
+      <c r="D347">
+        <v>0.72727272727272729</v>
+      </c>
+      <c r="E347" t="s">
+        <v>16</v>
+      </c>
+      <c r="F347">
+        <v>2.5</v>
+      </c>
+      <c r="G347">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="348" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A348" t="s">
+        <v>14</v>
+      </c>
+      <c r="B348" t="s">
+        <v>15</v>
+      </c>
+      <c r="C348">
+        <v>0.75238095238095237</v>
+      </c>
+      <c r="D348">
+        <v>0.56060606060606055</v>
+      </c>
+      <c r="E348" t="s">
+        <v>16</v>
+      </c>
+      <c r="F348">
+        <v>2.5</v>
+      </c>
+      <c r="G348">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="349" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A349" t="s">
+        <v>14</v>
+      </c>
+      <c r="B349" t="s">
+        <v>15</v>
+      </c>
+      <c r="C349">
+        <v>0.67738095238095253</v>
+      </c>
+      <c r="D349">
+        <v>0.81818181818181812</v>
+      </c>
+      <c r="E349" t="s">
+        <v>16</v>
+      </c>
+      <c r="F349">
+        <v>2.5</v>
+      </c>
+      <c r="G349">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="350" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A350" t="s">
+        <v>14</v>
+      </c>
+      <c r="B350" t="s">
+        <v>15</v>
+      </c>
+      <c r="C350">
+        <v>0.53650793650793649</v>
+      </c>
+      <c r="D350">
+        <v>0.77272727272727271</v>
+      </c>
+      <c r="E350" t="s">
+        <v>16</v>
+      </c>
+      <c r="F350">
+        <v>2.5</v>
+      </c>
+      <c r="G350">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="351" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A351" t="s">
+        <v>14</v>
+      </c>
+      <c r="B351" t="s">
+        <v>15</v>
+      </c>
+      <c r="C351">
+        <v>0.75952380952380949</v>
+      </c>
+      <c r="D351">
+        <v>0.81818181818181812</v>
+      </c>
+      <c r="E351" t="s">
+        <v>16</v>
+      </c>
+      <c r="F351">
+        <v>2.5</v>
+      </c>
+      <c r="G351">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="352" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A352" t="s">
+        <v>14</v>
+      </c>
+      <c r="B352" t="s">
+        <v>15</v>
+      </c>
+      <c r="C352">
+        <v>0.73174603174603181</v>
+      </c>
+      <c r="D352">
+        <v>0.90909090909090917</v>
+      </c>
+      <c r="E352" t="s">
+        <v>16</v>
+      </c>
+      <c r="F352">
+        <v>2.5</v>
+      </c>
+      <c r="G352">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="353" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A353" t="s">
+        <v>14</v>
+      </c>
+      <c r="B353" t="s">
+        <v>15</v>
+      </c>
+      <c r="C353">
+        <v>0.61865079365079367</v>
+      </c>
+      <c r="D353">
+        <v>0.86363636363636365</v>
+      </c>
+      <c r="E353" t="s">
+        <v>16</v>
+      </c>
+      <c r="F353">
+        <v>2.5</v>
+      </c>
+      <c r="G353">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="354" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A354" t="s">
+        <v>14</v>
+      </c>
+      <c r="B354" t="s">
+        <v>15</v>
+      </c>
+      <c r="C354">
+        <v>0.6880952380952382</v>
+      </c>
+      <c r="D354">
+        <v>0.62121212121212122</v>
+      </c>
+      <c r="E354" t="s">
+        <v>16</v>
+      </c>
+      <c r="F354">
+        <v>2.5</v>
+      </c>
+      <c r="G354">
+        <v>40</v>
+      </c>
+      <c r="H354" t="s">
+        <v>107</v>
+      </c>
+      <c r="I354" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="355" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A355" t="s">
+        <v>12</v>
+      </c>
+      <c r="B355" t="s">
+        <v>43</v>
+      </c>
+      <c r="C355">
+        <v>0.62698412698412698</v>
+      </c>
+      <c r="D355">
+        <v>0.5757575757575758</v>
+      </c>
+      <c r="E355" t="s">
+        <v>16</v>
+      </c>
+      <c r="F355">
+        <v>2.5</v>
+      </c>
+      <c r="G355">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="356" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A356" t="s">
+        <v>12</v>
+      </c>
+      <c r="B356" t="s">
+        <v>109</v>
+      </c>
+      <c r="C356">
+        <v>0.71507936507936509</v>
+      </c>
+      <c r="D356">
+        <v>0.53030303030303028</v>
+      </c>
+      <c r="E356" t="s">
+        <v>16</v>
+      </c>
+      <c r="F356">
+        <v>2.5</v>
+      </c>
+      <c r="G356">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="357" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A357" t="s">
+        <v>12</v>
+      </c>
+      <c r="B357" t="s">
+        <v>82</v>
+      </c>
+      <c r="C357">
+        <v>0.75396825396825395</v>
+      </c>
+      <c r="D357">
+        <v>0.62121212121212122</v>
+      </c>
+      <c r="E357" t="s">
+        <v>16</v>
+      </c>
+      <c r="F357">
+        <v>2.5</v>
+      </c>
+      <c r="G357">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="358" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A358" t="s">
+        <v>12</v>
+      </c>
+      <c r="B358" t="s">
+        <v>22</v>
+      </c>
+      <c r="C358">
+        <v>0.67063492063492058</v>
+      </c>
+      <c r="D358">
+        <v>0.69696969696969702</v>
+      </c>
+      <c r="E358" t="s">
+        <v>16</v>
+      </c>
+      <c r="F358">
+        <v>2.5</v>
+      </c>
+      <c r="G358">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="359" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A359" t="s">
+        <v>12</v>
+      </c>
+      <c r="B359" t="s">
+        <v>22</v>
+      </c>
+      <c r="C359">
+        <v>0.82341269841269848</v>
+      </c>
+      <c r="D359">
+        <v>0.5757575757575758</v>
+      </c>
+      <c r="E359" t="s">
+        <v>16</v>
+      </c>
+      <c r="F359">
+        <v>2.5</v>
+      </c>
+      <c r="G359">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="360" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A360" t="s">
+        <v>12</v>
+      </c>
+      <c r="B360" t="s">
+        <v>29</v>
+      </c>
+      <c r="C360">
+        <v>0.67539682539682533</v>
+      </c>
+      <c r="D360">
+        <v>0.74242424242424243</v>
+      </c>
+      <c r="E360" t="s">
+        <v>16</v>
+      </c>
+      <c r="F360">
+        <v>2.5</v>
+      </c>
+      <c r="G360">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="361" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A361" t="s">
+        <v>12</v>
+      </c>
+      <c r="B361" t="s">
+        <v>26</v>
+      </c>
+      <c r="C361">
+        <v>0.66349206349206347</v>
+      </c>
+      <c r="D361">
+        <v>0.53030303030303028</v>
+      </c>
+      <c r="E361" t="s">
+        <v>16</v>
+      </c>
+      <c r="F361">
+        <v>2.5</v>
+      </c>
+      <c r="G361">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="362" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A362" t="s">
+        <v>12</v>
+      </c>
+      <c r="B362" t="s">
+        <v>29</v>
+      </c>
+      <c r="C362">
+        <v>0.59285714285714286</v>
+      </c>
+      <c r="D362">
+        <v>0.78787878787878785</v>
+      </c>
+      <c r="E362" t="s">
+        <v>16</v>
+      </c>
+      <c r="F362">
+        <v>2.5</v>
+      </c>
+      <c r="G362">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="363" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A363" t="s">
+        <v>12</v>
+      </c>
+      <c r="B363" t="s">
+        <v>110</v>
+      </c>
+      <c r="C363">
+        <v>0.71230158730158732</v>
+      </c>
+      <c r="D363">
+        <v>0.53030303030303028</v>
+      </c>
+      <c r="E363" t="s">
+        <v>16</v>
+      </c>
+      <c r="F363">
+        <v>2.5</v>
+      </c>
+      <c r="G363">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="364" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A364" t="s">
+        <v>12</v>
+      </c>
+      <c r="B364" t="s">
+        <v>37</v>
+      </c>
+      <c r="C364">
+        <v>0.72896825396825404</v>
+      </c>
+      <c r="D364">
+        <v>0.72727272727272729</v>
+      </c>
+      <c r="E364" t="s">
+        <v>16</v>
+      </c>
+      <c r="F364">
+        <v>2.5</v>
+      </c>
+      <c r="G364">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="365" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A365" t="s">
+        <v>12</v>
+      </c>
+      <c r="B365" t="s">
+        <v>29</v>
+      </c>
+      <c r="C365">
+        <v>0.60317460317460314</v>
+      </c>
+      <c r="D365">
+        <v>0.62121212121212122</v>
+      </c>
+      <c r="E365" t="s">
+        <v>16</v>
+      </c>
+      <c r="F365">
+        <v>2.5</v>
+      </c>
+      <c r="G365">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="366" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A366" t="s">
+        <v>12</v>
+      </c>
+      <c r="B366" t="s">
+        <v>35</v>
+      </c>
+      <c r="C366">
+        <v>0.71587301587301588</v>
+      </c>
+      <c r="D366">
+        <v>0.65151515151515149</v>
+      </c>
+      <c r="E366" t="s">
+        <v>16</v>
+      </c>
+      <c r="F366">
+        <v>2.5</v>
+      </c>
+      <c r="G366">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="367" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A367" t="s">
+        <v>12</v>
+      </c>
+      <c r="B367" t="s">
+        <v>83</v>
+      </c>
+      <c r="C367">
+        <v>0.65476190476190477</v>
+      </c>
+      <c r="D367">
+        <v>0.5757575757575758</v>
+      </c>
+      <c r="E367" t="s">
+        <v>16</v>
+      </c>
+      <c r="F367">
+        <v>2.5</v>
+      </c>
+      <c r="G367">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="368" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A368" t="s">
+        <v>12</v>
+      </c>
+      <c r="B368" t="s">
+        <v>25</v>
+      </c>
+      <c r="C368">
+        <v>0.69761904761904747</v>
+      </c>
+      <c r="D368">
+        <v>0.62121212121212122</v>
+      </c>
+      <c r="E368" t="s">
+        <v>16</v>
+      </c>
+      <c r="F368">
+        <v>2.5</v>
+      </c>
+      <c r="G368">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="369" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A369" t="s">
+        <v>12</v>
+      </c>
+      <c r="B369" t="s">
+        <v>80</v>
+      </c>
+      <c r="C369">
+        <v>0.80753968253968245</v>
+      </c>
+      <c r="D369">
+        <v>0.74242424242424243</v>
+      </c>
+      <c r="E369" t="s">
+        <v>16</v>
+      </c>
+      <c r="F369">
+        <v>2.5</v>
+      </c>
+      <c r="G369">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="370" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A370" t="s">
+        <v>12</v>
+      </c>
+      <c r="B370" t="s">
+        <v>24</v>
+      </c>
+      <c r="C370">
+        <v>0.58611111111111114</v>
+      </c>
+      <c r="D370">
+        <v>0.74242424242424243</v>
+      </c>
+      <c r="E370" t="s">
+        <v>16</v>
+      </c>
+      <c r="F370">
+        <v>2.5</v>
+      </c>
+      <c r="G370">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="371" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A371" t="s">
+        <v>12</v>
+      </c>
+      <c r="B371" t="s">
+        <v>21</v>
+      </c>
+      <c r="C371">
+        <v>0.63888888888888884</v>
+      </c>
+      <c r="D371">
+        <v>0.48484848484848492</v>
+      </c>
+      <c r="E371" t="s">
+        <v>16</v>
+      </c>
+      <c r="F371">
+        <v>2.5</v>
+      </c>
+      <c r="G371">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="372" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A372" t="s">
+        <v>12</v>
+      </c>
+      <c r="B372" t="s">
+        <v>109</v>
+      </c>
+      <c r="C372">
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="D372">
+        <v>0.45454545454545447</v>
+      </c>
+      <c r="E372" t="s">
+        <v>16</v>
+      </c>
+      <c r="F372">
+        <v>2.5</v>
+      </c>
+      <c r="G372">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="373" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A373" t="s">
+        <v>12</v>
+      </c>
+      <c r="B373" t="s">
+        <v>38</v>
+      </c>
+      <c r="C373">
+        <v>0.74682539682539684</v>
+      </c>
+      <c r="D373">
+        <v>0.86363636363636365</v>
+      </c>
+      <c r="E373" t="s">
+        <v>16</v>
+      </c>
+      <c r="F373">
+        <v>2.5</v>
+      </c>
+      <c r="G373">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="374" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A374" t="s">
+        <v>12</v>
+      </c>
+      <c r="B374" t="s">
+        <v>38</v>
+      </c>
+      <c r="C374">
+        <v>0.8928571428571429</v>
+      </c>
+      <c r="D374">
+        <v>0.36363636363636359</v>
+      </c>
+      <c r="E374" t="s">
+        <v>16</v>
+      </c>
+      <c r="F374">
+        <v>2.5</v>
+      </c>
+      <c r="G374">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="375" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A375" t="s">
+        <v>12</v>
+      </c>
+      <c r="B375" t="s">
+        <v>40</v>
+      </c>
+      <c r="C375">
+        <v>0.69285714285714295</v>
+      </c>
+      <c r="D375">
+        <v>0.69696969696969702</v>
+      </c>
+      <c r="E375" t="s">
+        <v>16</v>
+      </c>
+      <c r="F375">
+        <v>2.5</v>
+      </c>
+      <c r="G375">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="376" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A376" t="s">
+        <v>12</v>
+      </c>
+      <c r="B376" t="s">
+        <v>111</v>
+      </c>
+      <c r="C376">
+        <v>0.57420634920634928</v>
+      </c>
+      <c r="D376">
+        <v>0.90909090909090917</v>
+      </c>
+      <c r="E376" t="s">
+        <v>16</v>
+      </c>
+      <c r="F376">
+        <v>2.5</v>
+      </c>
+      <c r="G376">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="377" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A377" t="s">
+        <v>12</v>
+      </c>
+      <c r="B377" t="s">
+        <v>82</v>
+      </c>
+      <c r="C377">
+        <v>0.74285714285714288</v>
+      </c>
+      <c r="D377">
+        <v>0.36363636363636359</v>
+      </c>
+      <c r="E377" t="s">
+        <v>16</v>
+      </c>
+      <c r="F377">
+        <v>2.5</v>
+      </c>
+      <c r="G377">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="378" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A378" t="s">
+        <v>12</v>
+      </c>
+      <c r="B378" t="s">
+        <v>112</v>
+      </c>
+      <c r="C378">
+        <v>0.72896825396825393</v>
+      </c>
+      <c r="D378">
+        <v>0.83333333333333326</v>
+      </c>
+      <c r="E378" t="s">
+        <v>16</v>
+      </c>
+      <c r="F378">
+        <v>2.5</v>
+      </c>
+      <c r="G378">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="379" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A379" t="s">
+        <v>12</v>
+      </c>
+      <c r="B379" t="s">
+        <v>37</v>
+      </c>
+      <c r="C379">
+        <v>0.67817460317460332</v>
+      </c>
+      <c r="D379">
+        <v>0.48484848484848492</v>
+      </c>
+      <c r="E379" t="s">
+        <v>16</v>
+      </c>
+      <c r="F379">
+        <v>2.5</v>
+      </c>
+      <c r="G379">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="380" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A380" t="s">
+        <v>12</v>
+      </c>
+      <c r="B380" t="s">
+        <v>22</v>
+      </c>
+      <c r="C380">
+        <v>0.76507936507936503</v>
+      </c>
+      <c r="D380">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="E380" t="s">
+        <v>16</v>
+      </c>
+      <c r="F380">
+        <v>2.5</v>
+      </c>
+      <c r="G380">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="381" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A381" t="s">
+        <v>12</v>
+      </c>
+      <c r="B381" t="s">
+        <v>113</v>
+      </c>
+      <c r="C381">
+        <v>0.81587301587301597</v>
+      </c>
+      <c r="D381">
+        <v>0.5757575757575758</v>
+      </c>
+      <c r="E381" t="s">
+        <v>16</v>
+      </c>
+      <c r="F381">
+        <v>2.5</v>
+      </c>
+      <c r="G381">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="382" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A382" t="s">
+        <v>12</v>
+      </c>
+      <c r="B382" t="s">
+        <v>24</v>
+      </c>
+      <c r="C382">
+        <v>0.73333333333333339</v>
+      </c>
+      <c r="D382">
+        <v>0.60606060606060597</v>
+      </c>
+      <c r="E382" t="s">
+        <v>16</v>
+      </c>
+      <c r="F382">
+        <v>2.5</v>
+      </c>
+      <c r="G382">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="383" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A383" t="s">
+        <v>12</v>
+      </c>
+      <c r="B383" t="s">
+        <v>33</v>
+      </c>
+      <c r="C383">
+        <v>0.74722222222222223</v>
+      </c>
+      <c r="D383">
+        <v>0.95454545454545459</v>
+      </c>
+      <c r="E383" t="s">
+        <v>16</v>
+      </c>
+      <c r="F383">
+        <v>2.5</v>
+      </c>
+      <c r="G383">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="384" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A384" t="s">
+        <v>12</v>
+      </c>
+      <c r="B384" t="s">
+        <v>13</v>
+      </c>
+      <c r="C384">
+        <v>0.71587301587301588</v>
+      </c>
+      <c r="D384">
+        <v>0.90909090909090917</v>
+      </c>
+      <c r="E384" t="s">
+        <v>16</v>
+      </c>
+      <c r="F384">
+        <v>2.5</v>
+      </c>
+      <c r="G384">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="385" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A385" t="s">
+        <v>12</v>
+      </c>
+      <c r="B385" t="s">
+        <v>37</v>
+      </c>
+      <c r="C385">
+        <v>0.70119047619047625</v>
+      </c>
+      <c r="D385">
+        <v>0.77272727272727271</v>
+      </c>
+      <c r="E385" t="s">
+        <v>16</v>
+      </c>
+      <c r="F385">
+        <v>2.5</v>
+      </c>
+      <c r="G385">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="386" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A386" t="s">
+        <v>12</v>
+      </c>
+      <c r="B386" t="s">
+        <v>24</v>
+      </c>
+      <c r="C386">
+        <v>0.71785714285714286</v>
+      </c>
+      <c r="D386">
+        <v>1</v>
+      </c>
+      <c r="E386" t="s">
+        <v>16</v>
+      </c>
+      <c r="F386">
+        <v>2.5</v>
+      </c>
+      <c r="G386">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="387" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A387" t="s">
+        <v>12</v>
+      </c>
+      <c r="B387" t="s">
+        <v>29</v>
+      </c>
+      <c r="C387">
+        <v>0.62063492063492065</v>
+      </c>
+      <c r="D387">
+        <v>0.65151515151515149</v>
+      </c>
+      <c r="E387" t="s">
+        <v>16</v>
+      </c>
+      <c r="F387">
+        <v>2.5</v>
+      </c>
+      <c r="G387">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="388" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A388" t="s">
+        <v>12</v>
+      </c>
+      <c r="B388" t="s">
+        <v>40</v>
+      </c>
+      <c r="C388">
+        <v>0.79563492063492058</v>
+      </c>
+      <c r="D388">
+        <v>0.5757575757575758</v>
+      </c>
+      <c r="E388" t="s">
+        <v>16</v>
+      </c>
+      <c r="F388">
+        <v>2.5</v>
+      </c>
+      <c r="G388">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="389" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A389" t="s">
+        <v>12</v>
+      </c>
+      <c r="B389" t="s">
+        <v>34</v>
+      </c>
+      <c r="C389">
+        <v>0.81111111111111123</v>
+      </c>
+      <c r="D389">
+        <v>0.81818181818181812</v>
+      </c>
+      <c r="E389" t="s">
+        <v>16</v>
+      </c>
+      <c r="F389">
+        <v>2.5</v>
+      </c>
+      <c r="G389">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="390" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A390" t="s">
+        <v>12</v>
+      </c>
+      <c r="B390" t="s">
+        <v>38</v>
+      </c>
+      <c r="C390">
+        <v>0.70198412698412704</v>
+      </c>
+      <c r="D390">
+        <v>0.95454545454545459</v>
+      </c>
+      <c r="E390" t="s">
+        <v>16</v>
+      </c>
+      <c r="F390">
+        <v>2.5</v>
+      </c>
+      <c r="G390">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="391" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A391" t="s">
+        <v>12</v>
+      </c>
+      <c r="B391" t="s">
+        <v>28</v>
+      </c>
+      <c r="C391">
+        <v>0.71865079365079365</v>
+      </c>
+      <c r="D391">
+        <v>0.78787878787878785</v>
+      </c>
+      <c r="E391" t="s">
+        <v>16</v>
+      </c>
+      <c r="F391">
+        <v>2.5</v>
+      </c>
+      <c r="G391">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="392" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A392" t="s">
+        <v>12</v>
+      </c>
+      <c r="B392" t="s">
+        <v>114</v>
+      </c>
+      <c r="C392">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="D392">
+        <v>0.62121212121212122</v>
+      </c>
+      <c r="E392" t="s">
+        <v>16</v>
+      </c>
+      <c r="F392">
+        <v>2.5</v>
+      </c>
+      <c r="G392">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="393" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A393" t="s">
+        <v>12</v>
+      </c>
+      <c r="B393" t="s">
+        <v>38</v>
+      </c>
+      <c r="C393">
+        <v>0.76944444444444449</v>
+      </c>
+      <c r="D393">
+        <v>0.60606060606060597</v>
+      </c>
+      <c r="E393" t="s">
+        <v>16</v>
+      </c>
+      <c r="F393">
+        <v>2.5</v>
+      </c>
+      <c r="G393">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="394" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A394" t="s">
+        <v>12</v>
+      </c>
+      <c r="B394" t="s">
+        <v>109</v>
+      </c>
+      <c r="C394">
+        <v>0.64563492063492067</v>
+      </c>
+      <c r="D394">
+        <v>0.90909090909090917</v>
+      </c>
+      <c r="E394" t="s">
+        <v>16</v>
+      </c>
+      <c r="F394">
+        <v>2.5</v>
+      </c>
+      <c r="G394">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="395" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A395" t="s">
+        <v>12</v>
+      </c>
+      <c r="B395" t="s">
+        <v>26</v>
+      </c>
+      <c r="C395">
+        <v>0.75198412698412698</v>
+      </c>
+      <c r="D395">
+        <v>0.62121212121212122</v>
+      </c>
+      <c r="E395" t="s">
+        <v>16</v>
+      </c>
+      <c r="F395">
+        <v>2.5</v>
+      </c>
+      <c r="G395">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="396" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A396" t="s">
+        <v>12</v>
+      </c>
+      <c r="B396" t="s">
+        <v>34</v>
+      </c>
+      <c r="C396">
+        <v>0.79365079365079361</v>
+      </c>
+      <c r="D396">
+        <v>0.74242424242424243</v>
+      </c>
+      <c r="E396" t="s">
+        <v>16</v>
+      </c>
+      <c r="F396">
+        <v>2.5</v>
+      </c>
+      <c r="G396">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="397" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A397" t="s">
+        <v>12</v>
+      </c>
+      <c r="B397" t="s">
+        <v>29</v>
+      </c>
+      <c r="C397">
+        <v>0.73174603174603181</v>
+      </c>
+      <c r="D397">
+        <v>0.74242424242424243</v>
+      </c>
+      <c r="E397" t="s">
+        <v>16</v>
+      </c>
+      <c r="F397">
+        <v>2.5</v>
+      </c>
+      <c r="G397">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="398" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A398" t="s">
+        <v>12</v>
+      </c>
+      <c r="B398" t="s">
+        <v>37</v>
+      </c>
+      <c r="C398">
+        <v>0.79761904761904756</v>
+      </c>
+      <c r="D398">
+        <v>0.65151515151515149</v>
+      </c>
+      <c r="E398" t="s">
+        <v>16</v>
+      </c>
+      <c r="F398">
+        <v>2.5</v>
+      </c>
+      <c r="G398">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="399" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A399" t="s">
+        <v>12</v>
+      </c>
+      <c r="B399" t="s">
+        <v>37</v>
+      </c>
+      <c r="C399">
+        <v>0.63492063492063489</v>
+      </c>
+      <c r="D399">
+        <v>0.53030303030303028</v>
+      </c>
+      <c r="E399" t="s">
+        <v>16</v>
+      </c>
+      <c r="F399">
+        <v>2.5</v>
+      </c>
+      <c r="G399">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="400" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A400" t="s">
+        <v>12</v>
+      </c>
+      <c r="B400" t="s">
+        <v>43</v>
+      </c>
+      <c r="C400">
+        <v>0.50753968253968262</v>
+      </c>
+      <c r="D400">
+        <v>0.86363636363636365</v>
+      </c>
+      <c r="E400" t="s">
+        <v>16</v>
+      </c>
+      <c r="F400">
+        <v>2.5</v>
+      </c>
+      <c r="G400">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="401" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A401" t="s">
+        <v>12</v>
+      </c>
+      <c r="B401" t="s">
+        <v>38</v>
+      </c>
+      <c r="C401">
+        <v>0.68333333333333324</v>
+      </c>
+      <c r="D401">
+        <v>0.53030303030303028</v>
+      </c>
+      <c r="E401" t="s">
+        <v>16</v>
+      </c>
+      <c r="F401">
+        <v>2.5</v>
+      </c>
+      <c r="G401">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="402" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A402" t="s">
+        <v>12</v>
+      </c>
+      <c r="B402" t="s">
+        <v>37</v>
+      </c>
+      <c r="C402">
+        <v>0.78134920634920635</v>
+      </c>
+      <c r="D402">
+        <v>0.5</v>
+      </c>
+      <c r="E402" t="s">
+        <v>16</v>
+      </c>
+      <c r="F402">
+        <v>2.5</v>
+      </c>
+      <c r="G402">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="403" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A403" t="s">
+        <v>12</v>
+      </c>
+      <c r="B403" t="s">
+        <v>25</v>
+      </c>
+      <c r="C403">
+        <v>0.60198412698412707</v>
+      </c>
+      <c r="D403">
+        <v>0.74242424242424243</v>
+      </c>
+      <c r="E403" t="s">
+        <v>16</v>
+      </c>
+      <c r="F403">
+        <v>2.5</v>
+      </c>
+      <c r="G403">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="404" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A404" t="s">
+        <v>12</v>
+      </c>
+      <c r="B404" t="s">
+        <v>41</v>
+      </c>
+      <c r="C404">
+        <v>0.74206349206349209</v>
+      </c>
+      <c r="D404">
+        <v>0.62121212121212122</v>
+      </c>
+      <c r="E404" t="s">
+        <v>16</v>
+      </c>
+      <c r="F404">
+        <v>2.5</v>
+      </c>
+      <c r="G404">
+        <v>40</v>
+      </c>
+      <c r="H404" t="s">
+        <v>115</v>
+      </c>
+      <c r="I404" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="405" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A405" t="s">
+        <v>9</v>
+      </c>
+      <c r="B405" t="s">
+        <v>117</v>
+      </c>
+      <c r="C405">
+        <v>0.73888888888888893</v>
+      </c>
+      <c r="D405">
+        <v>0.65151515151515149</v>
+      </c>
+      <c r="E405" t="s">
+        <v>16</v>
+      </c>
+      <c r="F405">
+        <v>2.5</v>
+      </c>
+      <c r="G405">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="406" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A406" t="s">
+        <v>9</v>
+      </c>
+      <c r="B406" t="s">
+        <v>10</v>
+      </c>
+      <c r="C406">
+        <v>0.74444444444444446</v>
+      </c>
+      <c r="D406">
+        <v>0.36363636363636359</v>
+      </c>
+      <c r="E406" t="s">
+        <v>16</v>
+      </c>
+      <c r="F406">
+        <v>2.5</v>
+      </c>
+      <c r="G406">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="407" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A407" t="s">
+        <v>9</v>
+      </c>
+      <c r="B407" t="s">
+        <v>47</v>
+      </c>
+      <c r="C407">
+        <v>0.73492063492063497</v>
+      </c>
+      <c r="D407">
+        <v>0.39393939393939392</v>
+      </c>
+      <c r="E407" t="s">
+        <v>16</v>
+      </c>
+      <c r="F407">
+        <v>2.5</v>
+      </c>
+      <c r="G407">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="408" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A408" t="s">
+        <v>9</v>
+      </c>
+      <c r="B408" t="s">
+        <v>55</v>
+      </c>
+      <c r="C408">
+        <v>0.81349206349206338</v>
+      </c>
+      <c r="D408">
+        <v>0.48484848484848492</v>
+      </c>
+      <c r="E408" t="s">
+        <v>16</v>
+      </c>
+      <c r="F408">
+        <v>2.5</v>
+      </c>
+      <c r="G408">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="409" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A409" t="s">
+        <v>9</v>
+      </c>
+      <c r="B409" t="s">
+        <v>91</v>
+      </c>
+      <c r="C409">
+        <v>0.82539682539682546</v>
+      </c>
+      <c r="D409">
+        <v>0.69696969696969702</v>
+      </c>
+      <c r="E409" t="s">
+        <v>16</v>
+      </c>
+      <c r="F409">
+        <v>2.5</v>
+      </c>
+      <c r="G409">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="410" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A410" t="s">
+        <v>9</v>
+      </c>
+      <c r="B410" t="s">
+        <v>60</v>
+      </c>
+      <c r="C410">
+        <v>0.67619047619047612</v>
+      </c>
+      <c r="D410">
+        <v>0.45454545454545447</v>
+      </c>
+      <c r="E410" t="s">
+        <v>16</v>
+      </c>
+      <c r="F410">
+        <v>2.5</v>
+      </c>
+      <c r="G410">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="411" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A411" t="s">
+        <v>9</v>
+      </c>
+      <c r="B411" t="s">
+        <v>118</v>
+      </c>
+      <c r="C411">
+        <v>0.56626984126984126</v>
+      </c>
+      <c r="D411">
+        <v>0.60606060606060597</v>
+      </c>
+      <c r="E411" t="s">
+        <v>16</v>
+      </c>
+      <c r="F411">
+        <v>2.5</v>
+      </c>
+      <c r="G411">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="412" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A412" t="s">
+        <v>9</v>
+      </c>
+      <c r="B412" t="s">
+        <v>48</v>
+      </c>
+      <c r="C412">
+        <v>0.78015873015873016</v>
+      </c>
+      <c r="D412">
+        <v>0.86363636363636365</v>
+      </c>
+      <c r="E412" t="s">
+        <v>16</v>
+      </c>
+      <c r="F412">
+        <v>2.5</v>
+      </c>
+      <c r="G412">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="413" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A413" t="s">
+        <v>9</v>
+      </c>
+      <c r="B413" t="s">
+        <v>94</v>
+      </c>
+      <c r="C413">
+        <v>0.77936507936507937</v>
+      </c>
+      <c r="D413">
+        <v>0.60606060606060597</v>
+      </c>
+      <c r="E413" t="s">
+        <v>16</v>
+      </c>
+      <c r="F413">
+        <v>2.5</v>
+      </c>
+      <c r="G413">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="414" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A414" t="s">
+        <v>9</v>
+      </c>
+      <c r="B414" t="s">
+        <v>51</v>
+      </c>
+      <c r="C414">
+        <v>0.77539682539682542</v>
+      </c>
+      <c r="D414">
+        <v>0.51515151515151514</v>
+      </c>
+      <c r="E414" t="s">
+        <v>16</v>
+      </c>
+      <c r="F414">
+        <v>2.5</v>
+      </c>
+      <c r="G414">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="415" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A415" t="s">
+        <v>9</v>
+      </c>
+      <c r="B415" t="s">
+        <v>50</v>
+      </c>
+      <c r="C415">
+        <v>0.66428571428571426</v>
+      </c>
+      <c r="D415">
+        <v>0.69696969696969702</v>
+      </c>
+      <c r="E415" t="s">
+        <v>16</v>
+      </c>
+      <c r="F415">
+        <v>2.5</v>
+      </c>
+      <c r="G415">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="416" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A416" t="s">
+        <v>9</v>
+      </c>
+      <c r="B416" t="s">
+        <v>67</v>
+      </c>
+      <c r="C416">
+        <v>0.68571428571428561</v>
+      </c>
+      <c r="D416">
+        <v>0.81818181818181812</v>
+      </c>
+      <c r="E416" t="s">
+        <v>16</v>
+      </c>
+      <c r="F416">
+        <v>2.5</v>
+      </c>
+      <c r="G416">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="417" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A417" t="s">
+        <v>9</v>
+      </c>
+      <c r="B417" t="s">
+        <v>88</v>
+      </c>
+      <c r="C417">
+        <v>0.73492063492063497</v>
+      </c>
+      <c r="D417">
+        <v>0.5757575757575758</v>
+      </c>
+      <c r="E417" t="s">
+        <v>16</v>
+      </c>
+      <c r="F417">
+        <v>2.5</v>
+      </c>
+      <c r="G417">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="418" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A418" t="s">
+        <v>9</v>
+      </c>
+      <c r="B418" t="s">
+        <v>63</v>
+      </c>
+      <c r="C418">
+        <v>0.61944444444444446</v>
+      </c>
+      <c r="D418">
+        <v>0.95454545454545459</v>
+      </c>
+      <c r="E418" t="s">
+        <v>16</v>
+      </c>
+      <c r="F418">
+        <v>2.5</v>
+      </c>
+      <c r="G418">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="419" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A419" t="s">
+        <v>9</v>
+      </c>
+      <c r="B419" t="s">
+        <v>48</v>
+      </c>
+      <c r="C419">
+        <v>0.7146825396825397</v>
+      </c>
+      <c r="D419">
+        <v>0.69696969696969702</v>
+      </c>
+      <c r="E419" t="s">
+        <v>16</v>
+      </c>
+      <c r="F419">
+        <v>2.5</v>
+      </c>
+      <c r="G419">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="420" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A420" t="s">
+        <v>9</v>
+      </c>
+      <c r="B420" t="s">
+        <v>103</v>
+      </c>
+      <c r="C420">
+        <v>0.73888888888888893</v>
+      </c>
+      <c r="D420">
+        <v>0.65151515151515149</v>
+      </c>
+      <c r="E420" t="s">
+        <v>16</v>
+      </c>
+      <c r="F420">
+        <v>2.5</v>
+      </c>
+      <c r="G420">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="421" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A421" t="s">
+        <v>9</v>
+      </c>
+      <c r="B421" t="s">
+        <v>48</v>
+      </c>
+      <c r="C421">
+        <v>0.76230158730158737</v>
+      </c>
+      <c r="D421">
+        <v>0.56060606060606055</v>
+      </c>
+      <c r="E421" t="s">
+        <v>16</v>
+      </c>
+      <c r="F421">
+        <v>2.5</v>
+      </c>
+      <c r="G421">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="422" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A422" t="s">
+        <v>9</v>
+      </c>
+      <c r="B422" t="s">
+        <v>72</v>
+      </c>
+      <c r="C422">
+        <v>0.84523809523809523</v>
+      </c>
+      <c r="D422">
+        <v>0.36363636363636359</v>
+      </c>
+      <c r="E422" t="s">
+        <v>16</v>
+      </c>
+      <c r="F422">
+        <v>2.5</v>
+      </c>
+      <c r="G422">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="423" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A423" t="s">
+        <v>9</v>
+      </c>
+      <c r="B423" t="s">
+        <v>52</v>
+      </c>
+      <c r="C423">
+        <v>0.64126984126984132</v>
+      </c>
+      <c r="D423">
+        <v>0.86363636363636365</v>
+      </c>
+      <c r="E423" t="s">
+        <v>16</v>
+      </c>
+      <c r="F423">
+        <v>2.5</v>
+      </c>
+      <c r="G423">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="424" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A424" t="s">
+        <v>9</v>
+      </c>
+      <c r="B424" t="s">
+        <v>72</v>
+      </c>
+      <c r="C424">
+        <v>0.70873015873015877</v>
+      </c>
+      <c r="D424">
+        <v>0.48484848484848492</v>
+      </c>
+      <c r="E424" t="s">
+        <v>16</v>
+      </c>
+      <c r="F424">
+        <v>2.5</v>
+      </c>
+      <c r="G424">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="425" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A425" t="s">
+        <v>9</v>
+      </c>
+      <c r="B425" t="s">
+        <v>72</v>
+      </c>
+      <c r="C425">
+        <v>0.71666666666666679</v>
+      </c>
+      <c r="D425">
+        <v>1</v>
+      </c>
+      <c r="E425" t="s">
+        <v>16</v>
+      </c>
+      <c r="F425">
+        <v>2.5</v>
+      </c>
+      <c r="G425">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="426" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A426" t="s">
+        <v>9</v>
+      </c>
+      <c r="B426" t="s">
+        <v>119</v>
+      </c>
+      <c r="C426">
+        <v>0.61388888888888882</v>
+      </c>
+      <c r="D426">
+        <v>0.65151515151515149</v>
+      </c>
+      <c r="E426" t="s">
+        <v>16</v>
+      </c>
+      <c r="F426">
+        <v>2.5</v>
+      </c>
+      <c r="G426">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="427" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A427" t="s">
+        <v>9</v>
+      </c>
+      <c r="B427" t="s">
+        <v>52</v>
+      </c>
+      <c r="C427">
+        <v>0.70317460317460323</v>
+      </c>
+      <c r="D427">
+        <v>0.27272727272727271</v>
+      </c>
+      <c r="E427" t="s">
+        <v>16</v>
+      </c>
+      <c r="F427">
+        <v>2.5</v>
+      </c>
+      <c r="G427">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="428" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A428" t="s">
+        <v>9</v>
+      </c>
+      <c r="B428" t="s">
+        <v>50</v>
+      </c>
+      <c r="C428">
+        <v>0.66587301587301584</v>
+      </c>
+      <c r="D428">
+        <v>0.77272727272727271</v>
+      </c>
+      <c r="E428" t="s">
+        <v>16</v>
+      </c>
+      <c r="F428">
+        <v>2.5</v>
+      </c>
+      <c r="G428">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="429" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A429" t="s">
+        <v>9</v>
+      </c>
+      <c r="B429" t="s">
+        <v>70</v>
+      </c>
+      <c r="C429">
+        <v>0.64841269841269844</v>
+      </c>
+      <c r="D429">
+        <v>0.53030303030303028</v>
+      </c>
+      <c r="E429" t="s">
+        <v>16</v>
+      </c>
+      <c r="F429">
+        <v>2.5</v>
+      </c>
+      <c r="G429">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="430" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A430" t="s">
+        <v>9</v>
+      </c>
+      <c r="B430" t="s">
+        <v>58</v>
+      </c>
+      <c r="C430">
+        <v>0.58690476190476193</v>
+      </c>
+      <c r="D430">
+        <v>0.90909090909090917</v>
+      </c>
+      <c r="E430" t="s">
+        <v>16</v>
+      </c>
+      <c r="F430">
+        <v>2.5</v>
+      </c>
+      <c r="G430">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="431" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A431" t="s">
+        <v>9</v>
+      </c>
+      <c r="B431" t="s">
+        <v>59</v>
+      </c>
+      <c r="C431">
+        <v>0.67896825396825411</v>
+      </c>
+      <c r="D431">
+        <v>0.90909090909090917</v>
+      </c>
+      <c r="E431" t="s">
+        <v>16</v>
+      </c>
+      <c r="F431">
+        <v>2.5</v>
+      </c>
+      <c r="G431">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="432" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A432" t="s">
+        <v>9</v>
+      </c>
+      <c r="B432" t="s">
+        <v>64</v>
+      </c>
+      <c r="C432">
+        <v>0.66547619047619044</v>
+      </c>
+      <c r="D432">
+        <v>0.51515151515151514</v>
+      </c>
+      <c r="E432" t="s">
+        <v>16</v>
+      </c>
+      <c r="F432">
+        <v>2.5</v>
+      </c>
+      <c r="G432">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="433" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A433" t="s">
+        <v>9</v>
+      </c>
+      <c r="B433" t="s">
+        <v>87</v>
+      </c>
+      <c r="C433">
+        <v>0.65634920634920635</v>
+      </c>
+      <c r="D433">
+        <v>0.78787878787878785</v>
+      </c>
+      <c r="E433" t="s">
+        <v>16</v>
+      </c>
+      <c r="F433">
+        <v>2.5</v>
+      </c>
+      <c r="G433">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="434" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A434" t="s">
+        <v>9</v>
+      </c>
+      <c r="B434" t="s">
+        <v>53</v>
+      </c>
+      <c r="C434">
+        <v>0.79246031746031742</v>
+      </c>
+      <c r="D434">
+        <v>0.77272727272727271</v>
+      </c>
+      <c r="E434" t="s">
+        <v>16</v>
+      </c>
+      <c r="F434">
+        <v>2.5</v>
+      </c>
+      <c r="G434">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="435" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A435" t="s">
+        <v>9</v>
+      </c>
+      <c r="B435" t="s">
+        <v>120</v>
+      </c>
+      <c r="C435">
+        <v>0.77460317460317463</v>
+      </c>
+      <c r="D435">
+        <v>0.60606060606060597</v>
+      </c>
+      <c r="E435" t="s">
+        <v>16</v>
+      </c>
+      <c r="F435">
+        <v>2.5</v>
+      </c>
+      <c r="G435">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="436" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A436" t="s">
+        <v>9</v>
+      </c>
+      <c r="B436" t="s">
+        <v>50</v>
+      </c>
+      <c r="C436">
+        <v>0.74285714285714288</v>
+      </c>
+      <c r="D436">
+        <v>0.65151515151515149</v>
+      </c>
+      <c r="E436" t="s">
+        <v>16</v>
+      </c>
+      <c r="F436">
+        <v>2.5</v>
+      </c>
+      <c r="G436">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="437" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A437" t="s">
+        <v>9</v>
+      </c>
+      <c r="B437" t="s">
+        <v>121</v>
+      </c>
+      <c r="C437">
+        <v>0.64484126984126977</v>
+      </c>
+      <c r="D437">
+        <v>0.81818181818181812</v>
+      </c>
+      <c r="E437" t="s">
+        <v>16</v>
+      </c>
+      <c r="F437">
+        <v>2.5</v>
+      </c>
+      <c r="G437">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="438" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A438" t="s">
+        <v>9</v>
+      </c>
+      <c r="B438" t="s">
+        <v>58</v>
+      </c>
+      <c r="C438">
+        <v>0.77460317460317463</v>
+      </c>
+      <c r="D438">
+        <v>0.78787878787878785</v>
+      </c>
+      <c r="E438" t="s">
+        <v>16</v>
+      </c>
+      <c r="F438">
+        <v>2.5</v>
+      </c>
+      <c r="G438">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="439" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A439" t="s">
+        <v>9</v>
+      </c>
+      <c r="B439" t="s">
+        <v>10</v>
+      </c>
+      <c r="C439">
+        <v>0.78373015873015872</v>
+      </c>
+      <c r="D439">
+        <v>0.86363636363636365</v>
+      </c>
+      <c r="E439" t="s">
+        <v>16</v>
+      </c>
+      <c r="F439">
+        <v>2.5</v>
+      </c>
+      <c r="G439">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="440" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A440" t="s">
+        <v>9</v>
+      </c>
+      <c r="B440" t="s">
+        <v>71</v>
+      </c>
+      <c r="C440">
+        <v>0.65952380952380951</v>
+      </c>
+      <c r="D440">
+        <v>0.86363636363636365</v>
+      </c>
+      <c r="E440" t="s">
+        <v>16</v>
+      </c>
+      <c r="F440">
+        <v>2.5</v>
+      </c>
+      <c r="G440">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="441" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A441" t="s">
+        <v>9</v>
+      </c>
+      <c r="B441" t="s">
+        <v>122</v>
+      </c>
+      <c r="C441">
+        <v>0.71309523809523812</v>
+      </c>
+      <c r="D441">
+        <v>0.69696969696969702</v>
+      </c>
+      <c r="E441" t="s">
+        <v>16</v>
+      </c>
+      <c r="F441">
+        <v>2.5</v>
+      </c>
+      <c r="G441">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="442" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A442" t="s">
+        <v>9</v>
+      </c>
+      <c r="B442" t="s">
+        <v>72</v>
+      </c>
+      <c r="C442">
+        <v>0.66349206349206347</v>
+      </c>
+      <c r="D442">
+        <v>0.90909090909090917</v>
+      </c>
+      <c r="E442" t="s">
+        <v>16</v>
+      </c>
+      <c r="F442">
+        <v>2.5</v>
+      </c>
+      <c r="G442">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="443" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A443" t="s">
+        <v>9</v>
+      </c>
+      <c r="B443" t="s">
+        <v>10</v>
+      </c>
+      <c r="C443">
+        <v>0.76428571428571435</v>
+      </c>
+      <c r="D443">
+        <v>0.65151515151515149</v>
+      </c>
+      <c r="E443" t="s">
+        <v>16</v>
+      </c>
+      <c r="F443">
+        <v>2.5</v>
+      </c>
+      <c r="G443">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="444" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A444" t="s">
+        <v>9</v>
+      </c>
+      <c r="B444" t="s">
+        <v>58</v>
+      </c>
+      <c r="C444">
+        <v>0.63650793650793647</v>
+      </c>
+      <c r="D444">
+        <v>0.78787878787878785</v>
+      </c>
+      <c r="E444" t="s">
+        <v>16</v>
+      </c>
+      <c r="F444">
+        <v>2.5</v>
+      </c>
+      <c r="G444">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="445" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A445" t="s">
+        <v>9</v>
+      </c>
+      <c r="B445" t="s">
+        <v>118</v>
+      </c>
+      <c r="C445">
+        <v>0.69761904761904769</v>
+      </c>
+      <c r="D445">
+        <v>0.78787878787878785</v>
+      </c>
+      <c r="E445" t="s">
+        <v>16</v>
+      </c>
+      <c r="F445">
+        <v>2.5</v>
+      </c>
+      <c r="G445">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="446" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A446" t="s">
+        <v>9</v>
+      </c>
+      <c r="B446" t="s">
+        <v>58</v>
+      </c>
+      <c r="C446">
+        <v>0.78452380952380951</v>
+      </c>
+      <c r="D446">
+        <v>0.53030303030303028</v>
+      </c>
+      <c r="E446" t="s">
+        <v>16</v>
+      </c>
+      <c r="F446">
+        <v>2.5</v>
+      </c>
+      <c r="G446">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="447" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A447" t="s">
+        <v>9</v>
+      </c>
+      <c r="B447" t="s">
+        <v>123</v>
+      </c>
+      <c r="C447">
+        <v>0.73015873015873023</v>
+      </c>
+      <c r="D447">
+        <v>0.81818181818181812</v>
+      </c>
+      <c r="E447" t="s">
+        <v>16</v>
+      </c>
+      <c r="F447">
+        <v>2.5</v>
+      </c>
+      <c r="G447">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="448" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A448" t="s">
+        <v>9</v>
+      </c>
+      <c r="B448" t="s">
+        <v>67</v>
+      </c>
+      <c r="C448">
+        <v>0.67023809523809519</v>
+      </c>
+      <c r="D448">
+        <v>0.86363636363636365</v>
+      </c>
+      <c r="E448" t="s">
+        <v>16</v>
+      </c>
+      <c r="F448">
+        <v>2.5</v>
+      </c>
+      <c r="G448">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="449" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A449" t="s">
+        <v>9</v>
+      </c>
+      <c r="B449" t="s">
+        <v>59</v>
+      </c>
+      <c r="C449">
+        <v>0.79047619047619044</v>
+      </c>
+      <c r="D449">
+        <v>0.81818181818181812</v>
+      </c>
+      <c r="E449" t="s">
+        <v>16</v>
+      </c>
+      <c r="F449">
+        <v>2.5</v>
+      </c>
+      <c r="G449">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="450" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A450" t="s">
+        <v>9</v>
+      </c>
+      <c r="B450" t="s">
+        <v>48</v>
+      </c>
+      <c r="C450">
+        <v>0.67738095238095253</v>
+      </c>
+      <c r="D450">
+        <v>0.65151515151515149</v>
+      </c>
+      <c r="E450" t="s">
+        <v>16</v>
+      </c>
+      <c r="F450">
+        <v>2.5</v>
+      </c>
+      <c r="G450">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="451" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A451" t="s">
+        <v>9</v>
+      </c>
+      <c r="B451" t="s">
+        <v>48</v>
+      </c>
+      <c r="C451">
+        <v>0.82619047619047625</v>
+      </c>
+      <c r="D451">
+        <v>0.48484848484848492</v>
+      </c>
+      <c r="E451" t="s">
+        <v>16</v>
+      </c>
+      <c r="F451">
+        <v>2.5</v>
+      </c>
+      <c r="G451">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="452" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A452" t="s">
+        <v>9</v>
+      </c>
+      <c r="B452" t="s">
+        <v>92</v>
+      </c>
+      <c r="C452">
+        <v>0.81190476190476202</v>
+      </c>
+      <c r="D452">
+        <v>0.62121212121212122</v>
+      </c>
+      <c r="E452" t="s">
+        <v>16</v>
+      </c>
+      <c r="F452">
+        <v>2.5</v>
+      </c>
+      <c r="G452">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="453" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A453" t="s">
+        <v>9</v>
+      </c>
+      <c r="B453" t="s">
+        <v>10</v>
+      </c>
+      <c r="C453">
+        <v>0.6880952380952382</v>
+      </c>
+      <c r="D453">
+        <v>0.77272727272727271</v>
+      </c>
+      <c r="E453" t="s">
+        <v>16</v>
+      </c>
+      <c r="F453">
+        <v>2.5</v>
+      </c>
+      <c r="G453">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="454" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A454" t="s">
+        <v>9</v>
+      </c>
+      <c r="B454" t="s">
+        <v>67</v>
+      </c>
+      <c r="C454">
+        <v>0.76468253968253974</v>
+      </c>
+      <c r="D454">
+        <v>0.95454545454545459</v>
+      </c>
+      <c r="E454" t="s">
+        <v>16</v>
+      </c>
+      <c r="F454">
+        <v>2.5</v>
+      </c>
+      <c r="G454">
+        <v>40</v>
+      </c>
+      <c r="H454" t="s">
+        <v>124</v>
+      </c>
+      <c r="I454" t="s">
+        <v>125</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Readme fixed + coherence results on alpha band
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://epflch-my.sharepoint.com/personal/martina_baroffio_epfl_ch/Documents/EPFL/MA1/ML/ML4Science/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_08C1AEB71759AA0F62355476585DCE3A874466E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3335836-0023-4678-AD19-6D4DE6904158}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_08C1AEB71759AA0F62355476585DCE3A874466E4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2165D0CB-84EE-401C-AC17-FB0B848A5B16}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -762,6 +762,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I454"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="80.7265625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">

</xml_diff>